<commit_message>
DCF: choose Gordon Growth or EBITDA exit multiple, mid-year option, user-entered assumptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company_analysis/output/company_analysis.xlsx
+++ b/company_analysis/output/company_analysis.xlsx
@@ -987,16 +987,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1035,6 +1037,16 @@
           <t>Value per share</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Implied exit multiple</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Implied terminal growth</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1051,16 +1063,20 @@
         <v>66987</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>1423981.439275594</v>
+        <v>2512183.6188039</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>1404622.439275594</v>
+        <v>2492824.6188039</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.7711848014993077</v>
+        <v>0.8645898976929792</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>188.4640331779946</v>
+        <v>334.4726444121696</v>
+      </c>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="3" t="n">
+        <v>0.0588157242301823</v>
       </c>
     </row>
     <row r="3">
@@ -1078,16 +1094,20 @@
         <v>73266</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>1557457.777329417</v>
+        <v>2092999.016093614</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1539080.777329417</v>
+        <v>2074622.016093614</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.7711848014993078</v>
+        <v>0.8222353612521957</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>125.8447078764855</v>
+        <v>169.633852501522</v>
+      </c>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="3" t="n">
+        <v>0.04741634432958686</v>
       </c>
     </row>
     <row r="4">
@@ -1105,16 +1125,20 @@
         <v>7695</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>163577.0698079582</v>
+        <v>1709088.504818912</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>181551.0698079582</v>
+        <v>1727062.504818912</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.7711848014993077</v>
+        <v>0.9771358011685451</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>16.76836333314475</v>
+        <v>159.5144088684688</v>
+      </c>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="3" t="n">
+        <v>0.08522476084093809</v>
       </c>
     </row>
     <row r="5">
@@ -1132,16 +1156,20 @@
         <v>46109</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>980165.7065334821</v>
+        <v>1401788.252415996</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>957294.7065334821</v>
+        <v>1378917.252415996</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.7711848014993077</v>
+        <v>0.8329620295679214</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>371.9093653976232</v>
+        <v>535.7098882735025</v>
+      </c>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="3" t="n">
+        <v>0.05038911171307355</v>
       </c>
     </row>
     <row r="6">
@@ -1159,16 +1187,20 @@
         <v>96676</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2055097.699903075</v>
+        <v>2017698.19601367</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2057234.699903075</v>
+        <v>2019835.19601367</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.7711848014993078</v>
+        <v>0.7566819179444675</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>83.92080851362793</v>
+        <v>82.3951699442633</v>
+      </c>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="3" t="n">
+        <v>0.02784676036134658</v>
       </c>
     </row>
     <row r="7">
@@ -1186,16 +1218,20 @@
         <v>7246</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>154032.4168717953</v>
+        <v>136792.8428619023</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>161259.4168717953</v>
+        <v>144019.8428619023</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.7711848014993079</v>
+        <v>0.731003349916275</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>271.6372523135212</v>
+        <v>242.5976426836169</v>
+      </c>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="3" t="n">
+        <v>0.01945443827149467</v>
       </c>
     </row>
     <row r="8">
@@ -1213,16 +1249,20 @@
         <v>3266.959</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>69447.63877878326</v>
+        <v>31855.53730828218</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>69447.63877878326</v>
+        <v>31855.53730828218</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.7711848014993078</v>
+        <v>0.4792003705199653</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>672.0798769925549</v>
+        <v>308.2821240889008</v>
+      </c>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="3" t="n">
+        <v>-0.09496631194299834</v>
       </c>
     </row>
     <row r="9">
@@ -1240,16 +1280,20 @@
         <v>4547.458</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>96667.94733135257</v>
+        <v>112224.9290786009</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>86722.60133135256</v>
+        <v>102279.5830786009</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.7711848014993077</v>
+        <v>0.7942256330978634</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>111.1520621690013</v>
+        <v>131.0913925832865</v>
+      </c>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="3" t="n">
+        <v>0.03936066187115802</v>
       </c>
     </row>
     <row r="10">
@@ -1267,16 +1311,20 @@
         <v>477.76</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>10156.02090597142</v>
+        <v>113739.3862564594</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>10156.02090597142</v>
+        <v>113739.3862564594</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.7711848014993078</v>
+        <v>0.9786690193001348</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>11.31419129840353</v>
+        <v>126.7099768878924</v>
+      </c>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="3" t="n">
+        <v>0.0855506206713556</v>
       </c>
     </row>
     <row r="11">
@@ -1294,16 +1342,20 @@
         <v>1198.284</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>25472.6167014632</v>
+        <v>12217.29775255978</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>22342.7027014632</v>
+        <v>9087.383752559785</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.7711848014993078</v>
+        <v>0.5019229635904449</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>33.7561643688261</v>
+        <v>13.72954846746982</v>
+      </c>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="3" t="n">
+        <v>-0.08141644710214198</v>
       </c>
     </row>
     <row r="13">
@@ -1316,34 +1368,71 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>FCF growth, years 1-5</t>
+          <t>Terminal value method</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
-      <c r="C14" s="3" t="n">
-        <v>0.08</v>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>EBITDA exit multiple</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Discount rate</t>
+          <t>Projection years</t>
         </is>
       </c>
       <c r="B15" s="2" t="n"/>
-      <c r="C15" s="3" t="n">
-        <v>0.09</v>
+      <c r="C15" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Terminal growth</t>
+          <t>Growth rate (cash flow and EBITDA)</t>
         </is>
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="3" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Discount rate</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="3" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Mid-year convention</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Exit EV / EBITDA multiple</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="5" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify metrics, SEC loader, DCF and Excel export (identical results)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company_analysis/output/company_analysis.xlsx
+++ b/company_analysis/output/company_analysis.xlsx
@@ -71,17 +71,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,18 +450,18 @@
   <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -991,13 +991,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1366,72 +1366,66 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Terminal value method</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>EBITDA exit multiple</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Projection years</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n">
+      <c r="C15" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Growth rate (cash flow and EBITDA)</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="8" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Discount rate</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="8" t="n">
         <v>0.09</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Mid-year convention</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Exit EV / EBITDA multiple</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="9" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1449,11 +1443,11 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1750,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1925,25 +1919,25 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SEC EDGAR XBRL company facts (latest 10-K). $ in millions.</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Caution</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>SEC EDGAR XBRL company facts (latest 10-K). $ in millions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Caution</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Asset managers consolidate funds/insurance units, so their leverage and margins are not comparable to operating companies.</t>
         </is>

</xml_diff>

<commit_message>
Show clear messages when openpyxl is missing or the report is open in Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company_analysis/output/company_analysis.xlsx
+++ b/company_analysis/output/company_analysis.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -81,7 +81,6 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1063,21 +1062,21 @@
         <v>66987</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>2512183.6188039</v>
+        <v>1486680.26890368</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>2492824.6188039</v>
+        <v>1467321.26890368</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.8645898976929792</v>
+        <v>0.7711848014993077</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>334.4726444121696</v>
-      </c>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="3" t="n">
-        <v>0.0588157242301823</v>
-      </c>
+        <v>196.8765958545122</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>6.067118821127274</v>
+      </c>
+      <c r="I2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1094,21 +1093,21 @@
         <v>73266</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>2092999.016093614</v>
+        <v>1626033.657000567</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2074622.016093614</v>
+        <v>1607656.657000567</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.8222353612521957</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>169.633852501522</v>
-      </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="3" t="n">
-        <v>0.04741634432958686</v>
-      </c>
+        <v>131.4518934587545</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>8.375115698351923</v>
+      </c>
+      <c r="I3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1125,21 +1124,21 @@
         <v>7695</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>1709088.504818912</v>
+        <v>170779.4746624541</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1727062.504818912</v>
+        <v>188753.4746624541</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.9771358011685451</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>159.5144088684688</v>
-      </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="3" t="n">
-        <v>0.08522476084093809</v>
-      </c>
+        <v>17.43358960584226</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0.9064474957284312</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1156,21 +1155,21 @@
         <v>46109</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>1401788.252415996</v>
+        <v>1023323.040573242</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1378917.252415996</v>
+        <v>1000452.040573242</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.8329620295679214</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>535.7098882735025</v>
-      </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="3" t="n">
-        <v>0.05038911171307355</v>
-      </c>
+        <v>388.6760064387109</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>7.768400201520564</v>
+      </c>
+      <c r="I5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1187,21 +1186,21 @@
         <v>96676</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2017698.19601367</v>
+        <v>2145584.989274518</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2019835.19601367</v>
+        <v>2147721.989274518</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.7566819179444675</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>82.3951699442633</v>
-      </c>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="3" t="n">
-        <v>0.02784676036134658</v>
-      </c>
+        <v>87.61205797807447</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>12.45668893392379</v>
+      </c>
+      <c r="I6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1218,21 +1217,21 @@
         <v>7246</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>136792.8428619023</v>
+        <v>160814.5644449828</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>144019.8428619023</v>
+        <v>168041.5644449828</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.731003349916275</v>
+        <v>0.7711848014993079</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>242.5976426836169</v>
-      </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="3" t="n">
-        <v>0.01945443827149467</v>
-      </c>
+        <v>283.0616017704593</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>14.2550615020246</v>
+      </c>
+      <c r="I7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1249,21 +1248,21 @@
         <v>3266.959</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>31855.53730828218</v>
+        <v>72505.46351705996</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>31855.53730828218</v>
+        <v>72505.46351705996</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.4792003705199653</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>308.2821240889008</v>
-      </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="3" t="n">
-        <v>-0.09496631194299834</v>
-      </c>
+        <v>701.6719914273173</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>42.1012618238116</v>
+      </c>
+      <c r="I8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1280,21 +1279,21 @@
         <v>4547.458</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>112224.9290786009</v>
+        <v>100924.2999726542</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>102279.5830786009</v>
+        <v>90978.95397265423</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.7942256330978634</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>131.0913925832865</v>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="3" t="n">
-        <v>0.03936066187115802</v>
-      </c>
+        <v>116.6074148237436</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>10.03665429838501</v>
+      </c>
+      <c r="I9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1311,21 +1310,21 @@
         <v>477.76</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>113739.3862564594</v>
+        <v>10603.19711692451</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>113739.3862564594</v>
+        <v>10603.19711692451</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.9786690193001348</v>
+        <v>0.7711848014993077</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>126.7099768878924</v>
-      </c>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="3" t="n">
-        <v>0.0855506206713556</v>
-      </c>
+        <v>11.81236250557815</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.8443384622026127</v>
+      </c>
+      <c r="I10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1342,21 +1341,21 @@
         <v>1198.284</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>12217.29775255978</v>
+        <v>26594.19259472698</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>9087.383752559785</v>
+        <v>23464.27859472698</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.5019229635904449</v>
+        <v>0.7711848014993078</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>13.72954846746982</v>
-      </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="3" t="n">
-        <v>-0.08141644710214198</v>
-      </c>
+        <v>35.45068184556116</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>38.44156363527635</v>
+      </c>
+      <c r="I11" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1373,7 +1372,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EBITDA exit multiple</t>
+          <t>Gordon Growth</t>
         </is>
       </c>
     </row>
@@ -1422,11 +1421,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Exit EV / EBITDA multiple</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v>12</v>
+          <t>Terminal growth rate</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>